<commit_message>
added a new sheet in ALA-LansdowneSouth.xlsx to preprocess
</commit_message>
<xml_diff>
--- a/ALA-LansdowneSouth.xlsx
+++ b/ALA-LansdowneSouth.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lemon\Capstone-Project-B\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1816185-38F7-4C19-9AF1-D1AE8C5216E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD5B48ED-E4FC-4136-A51E-BA5CA7291006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3805,14 +3805,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" pivotButton="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -3837,7 +3837,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="HyeokIn Kwon" refreshedDate="46125.557408564811" refreshedVersion="8" recordCount="82" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="HyeokIn Kwon" refreshedDate="46125.563670138887" refreshedVersion="8" recordCount="82" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:GW83" sheet="records-2026-03-03"/>
   </cacheSource>
@@ -22877,29 +22877,29 @@
       <c r="A4" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="16">
         <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="17">
         <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="11" t="s">
         <v>1191</v>
       </c>
-      <c r="B6" s="13"/>
+      <c r="B6" s="17"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="18">
         <v>81</v>
       </c>
     </row>
@@ -22920,71 +22920,71 @@
       <c r="A14" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="16">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="13">
+      <c r="B15" s="17">
         <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="13">
+      <c r="B16" s="17">
         <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="13">
+      <c r="B17" s="17">
         <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="13">
+      <c r="B18" s="17">
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="13">
+      <c r="B19" s="17">
         <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B20" s="13">
+      <c r="B20" s="17">
         <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="13">
+      <c r="B21" s="17">
         <v>21</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="14" t="s">
+      <c r="A22" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B22" s="15">
+      <c r="B22" s="18">
         <v>81</v>
       </c>
     </row>
@@ -23022,12 +23022,12 @@
       <c r="B29" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="16"/>
-      <c r="H29" s="17"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="13"/>
+      <c r="G29" s="13"/>
+      <c r="H29" s="14"/>
     </row>
     <row r="30" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
@@ -23036,19 +23036,19 @@
       <c r="B30" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C30" s="18" t="s">
+      <c r="C30" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="D30" s="18" t="s">
+      <c r="D30" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E30" s="18" t="s">
+      <c r="E30" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="F30" s="18" t="s">
+      <c r="F30" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="G30" s="18" t="s">
+      <c r="G30" s="15" t="s">
         <v>1191</v>
       </c>
       <c r="H30" s="9" t="s">
@@ -23067,12 +23067,12 @@
       <c r="E31" s="20"/>
       <c r="F31" s="20"/>
       <c r="G31" s="20"/>
-      <c r="H31" s="11">
+      <c r="H31" s="16">
         <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="12" t="s">
+      <c r="A32" s="11" t="s">
         <v>9</v>
       </c>
       <c r="B32" s="21"/>
@@ -23083,12 +23083,12 @@
       <c r="E32" s="22"/>
       <c r="F32" s="22"/>
       <c r="G32" s="22"/>
-      <c r="H32" s="13">
+      <c r="H32" s="17">
         <v>17</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="12" t="s">
+      <c r="A33" s="11" t="s">
         <v>10</v>
       </c>
       <c r="B33" s="21"/>
@@ -23099,12 +23099,12 @@
         <v>1</v>
       </c>
       <c r="G33" s="22"/>
-      <c r="H33" s="13">
+      <c r="H33" s="17">
         <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="12" t="s">
+      <c r="A34" s="11" t="s">
         <v>11</v>
       </c>
       <c r="B34" s="21">
@@ -23121,12 +23121,12 @@
       </c>
       <c r="F34" s="22"/>
       <c r="G34" s="22"/>
-      <c r="H34" s="13">
+      <c r="H34" s="17">
         <v>29</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="12" t="s">
+      <c r="A35" s="11" t="s">
         <v>12</v>
       </c>
       <c r="B35" s="21"/>
@@ -23137,12 +23137,12 @@
       <c r="E35" s="22"/>
       <c r="F35" s="22"/>
       <c r="G35" s="22"/>
-      <c r="H35" s="13">
+      <c r="H35" s="17">
         <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="12" t="s">
+      <c r="A36" s="11" t="s">
         <v>13</v>
       </c>
       <c r="B36" s="21"/>
@@ -23153,12 +23153,12 @@
       <c r="E36" s="22"/>
       <c r="F36" s="22"/>
       <c r="G36" s="22"/>
-      <c r="H36" s="13">
+      <c r="H36" s="17">
         <v>6</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="12" t="s">
+      <c r="A37" s="11" t="s">
         <v>14</v>
       </c>
       <c r="B37" s="21"/>
@@ -23169,12 +23169,12 @@
       <c r="E37" s="22"/>
       <c r="F37" s="22"/>
       <c r="G37" s="22"/>
-      <c r="H37" s="13">
+      <c r="H37" s="17">
         <v>5</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="12" t="s">
+      <c r="A38" s="11" t="s">
         <v>15</v>
       </c>
       <c r="B38" s="21"/>
@@ -23185,12 +23185,12 @@
       </c>
       <c r="F38" s="22"/>
       <c r="G38" s="22"/>
-      <c r="H38" s="13">
+      <c r="H38" s="17">
         <v>21</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="14" t="s">
+      <c r="A39" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B39" s="23">
@@ -23209,7 +23209,7 @@
         <v>1</v>
       </c>
       <c r="G39" s="24"/>
-      <c r="H39" s="15">
+      <c r="H39" s="18">
         <v>81</v>
       </c>
     </row>
@@ -24214,207 +24214,207 @@
       <c r="A4" s="10">
         <v>1900</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="16">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="12">
+      <c r="A5" s="11">
         <v>1913</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="17">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="12">
+      <c r="A6" s="11">
         <v>1950</v>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="17">
         <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="12">
+      <c r="A7" s="11">
         <v>1952</v>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="17">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="12">
+      <c r="A8" s="11">
         <v>1954</v>
       </c>
-      <c r="B8" s="13">
+      <c r="B8" s="17">
         <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="12">
+      <c r="A9" s="11">
         <v>1955</v>
       </c>
-      <c r="B9" s="13">
+      <c r="B9" s="17">
         <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="12">
+      <c r="A10" s="11">
         <v>1956</v>
       </c>
-      <c r="B10" s="13">
+      <c r="B10" s="17">
         <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="12">
+      <c r="A11" s="11">
         <v>1963</v>
       </c>
-      <c r="B11" s="13">
+      <c r="B11" s="17">
         <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="12">
+      <c r="A12" s="11">
         <v>1967</v>
       </c>
-      <c r="B12" s="13">
+      <c r="B12" s="17">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="12">
+      <c r="A13" s="11">
         <v>1973</v>
       </c>
-      <c r="B13" s="13">
+      <c r="B13" s="17">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="12">
+      <c r="A14" s="11">
         <v>1974</v>
       </c>
-      <c r="B14" s="13">
+      <c r="B14" s="17">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="12">
+      <c r="A15" s="11">
         <v>1977</v>
       </c>
-      <c r="B15" s="13">
+      <c r="B15" s="17">
         <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="12">
+      <c r="A16" s="11">
         <v>1978</v>
       </c>
-      <c r="B16" s="13">
+      <c r="B16" s="17">
         <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="12">
+      <c r="A17" s="11">
         <v>1979</v>
       </c>
-      <c r="B17" s="13">
+      <c r="B17" s="17">
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="12">
+      <c r="A18" s="11">
         <v>1987</v>
       </c>
-      <c r="B18" s="13">
+      <c r="B18" s="17">
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="12">
+      <c r="A19" s="11">
         <v>1993</v>
       </c>
-      <c r="B19" s="13">
+      <c r="B19" s="17">
         <v>7</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="12">
+      <c r="A20" s="11">
         <v>1997</v>
       </c>
-      <c r="B20" s="13">
+      <c r="B20" s="17">
         <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="12">
+      <c r="A21" s="11">
         <v>2000</v>
       </c>
-      <c r="B21" s="13">
+      <c r="B21" s="17">
         <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="12">
+      <c r="A22" s="11">
         <v>2019</v>
       </c>
-      <c r="B22" s="13">
+      <c r="B22" s="17">
         <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="12">
+      <c r="A23" s="11">
         <v>2021</v>
       </c>
-      <c r="B23" s="13">
+      <c r="B23" s="17">
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="12">
+      <c r="A24" s="11">
         <v>2022</v>
       </c>
-      <c r="B24" s="13">
+      <c r="B24" s="17">
         <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="12">
+      <c r="A25" s="11">
         <v>2023</v>
       </c>
-      <c r="B25" s="13">
+      <c r="B25" s="17">
         <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="12">
+      <c r="A26" s="11">
         <v>2024</v>
       </c>
-      <c r="B26" s="13">
+      <c r="B26" s="17">
         <v>4</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="12">
+      <c r="A27" s="11">
         <v>2025</v>
       </c>
-      <c r="B27" s="13">
+      <c r="B27" s="17">
         <v>12</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="12">
+      <c r="A28" s="11">
         <v>2026</v>
       </c>
-      <c r="B28" s="13">
+      <c r="B28" s="17">
         <v>9</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="14" t="s">
+      <c r="A29" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B29" s="15">
+      <c r="B29" s="18">
         <v>81</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated SQL and xlsx files (ALA & Garrison)
</commit_message>
<xml_diff>
--- a/ALA-LansdowneSouth.xlsx
+++ b/ALA-LansdowneSouth.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lemon\Capstone-Project-B\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lemon\Capstone-Test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD5B48ED-E4FC-4136-A51E-BA5CA7291006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B86CB99-A5A0-4FFC-B47A-B31ADB3D1116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3837,7 +3837,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="HyeokIn Kwon" refreshedDate="46125.563670138887" refreshedVersion="8" recordCount="82" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="HyeokIn Kwon" refreshedDate="46125.771961921295" refreshedVersion="8" recordCount="82" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:GW83" sheet="records-2026-03-03"/>
   </cacheSource>
@@ -39269,6 +39269,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1747DDC-0E08-401C-8DCD-825C7A462001}">
   <dimension ref="A1:GW54"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="147" max="147" width="63" bestFit="1" customWidth="1"/>
+    <col min="148" max="148" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="167" max="167" width="29.7109375" bestFit="1" customWidth="1"/>
+    <col min="168" max="168" width="29.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:205" x14ac:dyDescent="0.25">
       <c r="A1" t="s">

</xml_diff>

<commit_message>
All species are set to be unique. Ignore duplicated inputs from scientific_name column
</commit_message>
<xml_diff>
--- a/ALA-LansdowneSouth.xlsx
+++ b/ALA-LansdowneSouth.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lemon\Capstone-Test\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lemon\Capstone-Project-B\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B86CB99-A5A0-4FFC-B47A-B31ADB3D1116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70B3861A-E321-4A0F-BAEF-B6D854FD39A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3837,7 +3837,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="HyeokIn Kwon" refreshedDate="46125.771961921295" refreshedVersion="8" recordCount="82" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="HyeokIn Kwon" refreshedDate="46131.584372106481" refreshedVersion="8" recordCount="82" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:GW83" sheet="records-2026-03-03"/>
   </cacheSource>

</xml_diff>